<commit_message>
corrigir placares como float
</commit_message>
<xml_diff>
--- a/data/condominio.xlsx
+++ b/data/condominio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedrohamacher\OneDrive\Documentos antigo\Projetos_jl\Streamlit\Dashboard Pelada\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="14_{CCCF2471-6899-4BEE-B69A-61EDE0174783}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{99989A48-6A86-496D-98FD-95C8B4F5248B}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="14_{CCCF2471-6899-4BEE-B69A-61EDE0174783}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{1FF58352-21FD-4CDD-AB1B-3891BF8C526A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7890" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="notas" sheetId="1" r:id="rId1"/>
@@ -47684,7 +47684,9 @@
       <c r="A295" s="1">
         <v>46176</v>
       </c>
-      <c r="B295" s="62"/>
+      <c r="B295" s="62">
+        <v>1</v>
+      </c>
       <c r="C295" s="8" t="s">
         <v>1</v>
       </c>
@@ -47703,8 +47705,12 @@
       <c r="H295" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="I295" s="9"/>
-      <c r="J295" s="10"/>
+      <c r="I295" s="9">
+        <v>0</v>
+      </c>
+      <c r="J295" s="10">
+        <v>0</v>
+      </c>
       <c r="K295" s="10" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
bug artilharia Joao Marcio
</commit_message>
<xml_diff>
--- a/data/condominio.xlsx
+++ b/data/condominio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedrohamacher\OneDrive\Documentos antigo\Projetos_jl\Streamlit\Dashboard Pelada\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="14_{CCCF2471-6899-4BEE-B69A-61EDE0174783}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{1FF58352-21FD-4CDD-AB1B-3891BF8C526A}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="14_{CCCF2471-6899-4BEE-B69A-61EDE0174783}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{1830A4E2-765F-47E2-8AC0-FDF695CE3D23}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7890" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7890" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="notas" sheetId="1" r:id="rId1"/>
@@ -49903,9 +49903,6 @@
       <c r="Z39">
         <v>1</v>
       </c>
-      <c r="CB39">
-        <v>4</v>
-      </c>
     </row>
     <row r="40" spans="1:88" x14ac:dyDescent="0.35">
       <c r="A40" t="s">

</xml_diff>